<commit_message>
Update released dataset references
</commit_message>
<xml_diff>
--- a/results/combined/formal_experiment1_experiment2_merged_summary.xlsx
+++ b/results/combined/formal_experiment1_experiment2_merged_summary.xlsx
@@ -2022,7 +2022,7 @@
     <row r="1">
       <c r="A1" s="9" t="inlineStr">
         <is>
-          <t>Exp2_HV: no LERD, mean(std), Wilcoxon alpha=0.05 vs MOA-NSGAII</t>
+          <t>Exp2_HV: mean(std), Wilcoxon alpha=0.05 vs MOA-NSGAII</t>
         </is>
       </c>
       <c r="B1" s="10" t="n"/>
@@ -2697,7 +2697,7 @@
     <row r="1">
       <c r="A1" s="9" t="inlineStr">
         <is>
-          <t>Exp2_IGD: no LERD, mean(std), Wilcoxon alpha=0.05 vs MOA-NSGAII</t>
+          <t>Exp2_IGD: mean(std), Wilcoxon alpha=0.05 vs MOA-NSGAII</t>
         </is>
       </c>
       <c r="B1" s="10" t="n"/>

</xml_diff>